<commit_message>
Initial commit: stock screener with fundamentals, screening, and reporting pipeline
</commit_message>
<xml_diff>
--- a/data/screened_stocks.xlsx
+++ b/data/screened_stocks.xlsx
@@ -654,26 +654,34 @@
           <t>Information Technology Services</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>2093.5</v>
-      </c>
-      <c r="F2" t="n">
-        <v>7574465806336</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>₹2,088.00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>$79.56 Billion</t>
+        </is>
       </c>
       <c r="G2" t="n">
         <v>15.384333</v>
       </c>
       <c r="H2" t="n">
-        <v>12.743036</v>
+        <v>12.776619</v>
       </c>
       <c r="I2" t="n">
         <v>136.08</v>
       </c>
-      <c r="J2" t="n">
-        <v>2657010000000</v>
-      </c>
-      <c r="K2" t="n">
-        <v>493590000000</v>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>$27.91 Billion</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>$5.18 Billion</t>
+        </is>
       </c>
       <c r="L2" t="n">
         <v>0.40307</v>
@@ -684,10 +692,16 @@
       <c r="N2" t="n">
         <v>0.48395002</v>
       </c>
-      <c r="O2" t="n">
-        <v>112829997056</v>
-      </c>
-      <c r="P2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>$1.19 Billion</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>$11.26 Billion</t>
+        </is>
+      </c>
       <c r="Q2" t="n">
         <v>10.389</v>
       </c>
@@ -703,20 +717,30 @@
       <c r="U2" t="n">
         <v>0.241</v>
       </c>
-      <c r="V2" t="n">
-        <v>3426.1</v>
-      </c>
-      <c r="W2" t="n">
-        <v>1976.8</v>
-      </c>
-      <c r="X2" t="n">
-        <v>2709.1707</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>1860</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>3841</v>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>₹3,426.10</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>₹1,976.80</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>₹2,709.17</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>₹1,860.00</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>₹3,841.00</t>
+        </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
@@ -755,7 +779,7 @@
 2023-10-01 00:00:00+05:30   3095.42
 2023-11-01 00:00:00+05:30   3204.63
 2023-12-01 00:00:00+05:30   3485.62
-2024-01-01 00:00:00+05:30   3530.76
+2024-01-01 00:00:00+05:30   3530.77
 2024-02-01 00:00:00+05:30   3789.05
 2024-03-01 00:00:00+05:30   3586.60
 2024-04-01 00:00:00+05:30   3535.11
@@ -798,7 +822,7 @@
         <v>0.02530388431494646</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.2086452659548318</v>
+        <v>0.2086452954558826</v>
       </c>
       <c r="AF2" t="n">
         <v>18.2864965</v>
@@ -824,22 +848,30 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="AL2" t="n">
-        <v>3841</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>1860</v>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>₹3,841.00</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>₹1,860.00</t>
+        </is>
       </c>
       <c r="AN2" t="inlineStr">
         <is>
           <t>analyst consensus</t>
         </is>
       </c>
-      <c r="AO2" t="n">
-        <v>1860</v>
-      </c>
-      <c r="AP2" t="n">
-        <v>1767</v>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>₹1,860.00</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>₹1,767.00</t>
+        </is>
       </c>
       <c r="AQ2" t="n">
         <v>70</v>
@@ -866,11 +898,15 @@
           <t>Internet Content &amp; Information</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>582.9</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1479647035392</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>$582.65</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>$1.48 Trillion</t>
+        </is>
       </c>
       <c r="G3" t="n">
         <v>21.18866</v>
@@ -881,11 +917,15 @@
       <c r="I3" t="n">
         <v>27.51</v>
       </c>
-      <c r="J3" t="n">
-        <v>214962000000</v>
-      </c>
-      <c r="K3" t="n">
-        <v>70587000000</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>$214.96 Billion</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>$70.59 Billion</t>
+        </is>
       </c>
       <c r="L3" t="n">
         <v>0.81941</v>
@@ -896,10 +936,16 @@
       <c r="N3" t="n">
         <v>0.32930002</v>
       </c>
-      <c r="O3" t="n">
-        <v>86769000448</v>
-      </c>
-      <c r="P3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>$86.77 Billion</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>$217.24 Billion</t>
+        </is>
+      </c>
       <c r="Q3" t="n">
         <v>35.608</v>
       </c>
@@ -915,20 +961,30 @@
       <c r="U3" t="n">
         <v>1.246</v>
       </c>
-      <c r="V3" t="n">
-        <v>796.25</v>
-      </c>
-      <c r="W3" t="n">
-        <v>520.26</v>
-      </c>
-      <c r="X3" t="n">
-        <v>828.16864</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>664.46</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1015</v>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>$796.25</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>$520.26</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>$828.17</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>$664.46</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>$1,015.00</t>
+        </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
@@ -1010,7 +1066,7 @@
         <v>0.07405690015740007</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.4197937255625021</v>
+        <v>0.419793663104257</v>
       </c>
       <c r="AF3" t="n">
         <v>18.2864965</v>
@@ -1036,22 +1092,30 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="AL3" t="n">
-        <v>1015</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>664.46</v>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>$1,015.00</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>$664.46</t>
+        </is>
       </c>
       <c r="AN3" t="inlineStr">
         <is>
           <t>analyst consensus</t>
         </is>
       </c>
-      <c r="AO3" t="n">
-        <v>553.75</v>
-      </c>
-      <c r="AP3" t="n">
-        <v>509.85</v>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>$553.52</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>$509.85</t>
+        </is>
       </c>
       <c r="AQ3" t="n">
         <v>30</v>

</xml_diff>